<commit_message>
QA automation suite: Order Management rework + multi-feature WIP
Order Management:
- API-first seed/teardown (order-seed.ts: productId resolve, CancelOrder teardown)
- ORD_TEARDOWN branch in playwright.config.ts + global-teardown
- gen/upload-order-results scripts, update-order-design; refreshed design.md + xlsx
- result sync to Lark: 1 PASS (TA-04) / 36 BLOCKED (Forbidden — account not in
  inventory_order_workflow pic list); see FIXME-PLAN.md
- bug-card create payloads (TA-03 cancel-after-approved, TA-05 search-no-filter)

Other features (WIP carried in tree): product-stock, spare-parts, dashboards,
customer-form-configuration, customer-appointment teardown, case-ticket spec,
wiki updates, per-feature playwright configs + result-upload scripts.

Tooling: ignore disposable probe-*.mjs scratch.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/08-Order/order-management-testcases.xlsx
+++ b/08-Order/order-management-testcases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="273">
   <si>
     <t>META</t>
   </si>
@@ -213,7 +213,7 @@
     <t>New order created with status "Create Order" · Order No in format ORD260614-##### appears in the Order list</t>
   </si>
   <si>
-    <t>Order status "Create Order" · logged in as PIC of the "ส่งคำขอ" (Request) step</t>
+    <t>The order created in the same TS-01 flow (Create Order state). API alt: seedOrder(SEED_ORDER). Logged in as PIC of the "ส่งคำขอ" (Request) step. Teardown: CancelOrder (TS-01 walks to Complete OS009 which is terminal — see FIXME-PLAN no-DeleteOrder gap).</t>
   </si>
   <si>
     <t>TS-01_TC-05</t>
@@ -357,7 +357,7 @@
     <t>Order reaches the final step "เสร็จสิ้น" (Complete, OS009) · all 9 steps show ✓ with timestamp+actor · status badge = เสร็จสิ้น (terminal success)</t>
   </si>
   <si>
-    <t>Order with a requester + next-step PIC</t>
+    <t>The order from the TS-01 flow (has a requester + next-step PIC). API alt: seedOrder(SEED_ORDER).</t>
   </si>
   <si>
     <t>TS-01_TC-13</t>
@@ -369,7 +369,7 @@
     <t>PIC taps the Advance button of the current step</t>
   </si>
   <si>
-    <t>Action: advance step (e.g. apiwat.rod advancing to ส่งคำขอ on ORD260610-00003)</t>
+    <t>Action: advance step (the seeded/created order)</t>
   </si>
   <si>
     <t>All accounts related to the order (requester + next-step PIC) receive a real-time in-app bell notification with text "{actor} ส่งถึงคุณ {Status Name} :: {Order ID}" (e.g. "apiwat.rod ส่งถึงคุณ ส่งคำขอ :: ORD260610-00003"). [PO ORD-Q6]</t>
@@ -426,7 +426,7 @@
     <t>All columns present: ORDER · DETAIL · BILL TO · SHIP TO · ITEMS · STATUS · CREATED · REQUEST BY</t>
   </si>
   <si>
-    <t>Order ORD260610-00004 exists in the system</t>
+    <t>API seed: seedOrder(SEED_ORDER_OOS) — create a fresh order (iPhone 17 Pro Screen item) via GraphQL CreateOrder; open via the seeded orderId (no pre-existing data). Teardown: CancelOrder.</t>
   </si>
   <si>
     <t>TS-02_TC-03</t>
@@ -438,13 +438,13 @@
     <t>Open the order detail (click the row)</t>
   </si>
   <si>
-    <t>Order: ORD260610-00004</t>
-  </si>
-  <si>
-    <t>Shows Order No + status badge + date + requester (apiwat.rod) + Print button + Bill card (Bill To/Billing Address/Ship To/Shipping Address/Ship By) + ORDER ITEMS + OPERATING PROCEDURE (9-step workflow)</t>
-  </si>
-  <si>
-    <t>Order contains item "iPhone 17 Pro Screen" that is out of stock</t>
+    <t>Order: &lt;seeded orderId&gt; · item iPhone 17 Pro Screen</t>
+  </si>
+  <si>
+    <t>Shows Order No + status badge + date + requester + Print button + Bill card (Bill To/Billing Address/Ship To/Shipping Address/Ship By) + ORDER ITEMS + OPERATING PROCEDURE (9-step workflow)</t>
+  </si>
+  <si>
+    <t>Same seeded order as VO-detail (iPhone 17 Pro Screen item). ENV_DEPENDENT: the Out of Stock badge appears only if that product’s stock = 0 in the QA env.</t>
   </si>
   <si>
     <t>TS-02_TC-04</t>
@@ -456,13 +456,13 @@
     <t>Open detail → view the ORDER ITEMS section</t>
   </si>
   <si>
-    <t>Item: iPhone 17 Pro Screen (stock=0)</t>
-  </si>
-  <si>
-    <t>Item "iPhone 17 Pro Screen" shows an "Out of Stock" badge (red) + Quantity + Price 25,500 Baht</t>
-  </si>
-  <si>
-    <t>Order with no comment yet</t>
+    <t>Item: iPhone 17 Pro Screen</t>
+  </si>
+  <si>
+    <t>Item "iPhone 17 Pro Screen" shows an "Out of Stock" badge (red) + Quantity + Price (env-dependent on stock = 0)</t>
+  </si>
+  <si>
+    <t>Same seeded order as VO-detail (fresh = no comments yet)</t>
   </si>
   <si>
     <t>TS-02_TC-05</t>
@@ -477,7 +477,7 @@
     <t>Box shows "No Comment" + a "Comment..." input + a "Comment" button</t>
   </si>
   <si>
-    <t>Any order · Chat box open</t>
+    <t>Same seeded order as VO-detail · Chat box open</t>
   </si>
   <si>
     <t>TS-02_TC-06</t>
@@ -495,7 +495,7 @@
     <t>Comment "รบกวนเร่งจัดส่งภายในวันนี้ครับ" appears in the box (replacing "No Comment") with author name + timestamp</t>
   </si>
   <si>
-    <t>Order whose current step "ได้รับการอนุมัติ" (Approved) has been idle &gt; 61 minutes (SLA for this step)</t>
+    <t>ENV_DEPENDENT: needs an order at OS003 (ได้รับการอนุมัติ) idle &gt; 61 min — cannot seed + wait 61 min in CI. Provide ORD_OVERDUE_ID env pointing at such an order, else the step is skipped.</t>
   </si>
   <si>
     <t>TS-02_TC-07</t>
@@ -513,7 +513,7 @@
     <t>Current step shows an "Overdue" badge (red) next to "Current Step" once elapsed time exceeds 61 minutes. Each step has its own SLA in minutes. [PO ORD-Q4]</t>
   </si>
   <si>
-    <t>A search is active (Clear Filters button visible)</t>
+    <t>A search is active via the seeded orderId from VO-detail (Clear Filters button visible)</t>
   </si>
   <si>
     <t>TS-02_TC-08</t>
@@ -539,7 +539,7 @@
 3. Edit Title</t>
   </si>
   <si>
-    <t>Order with status "Create Order" (not yet submitted)</t>
+    <t>API seed: seedOrder(SEED_ORDER) — fresh order in Create Order state (OS000); open via the seeded orderId. Teardown: CancelOrder.</t>
   </si>
   <si>
     <t>TS-03_TC-01</t>
@@ -557,7 +557,7 @@
     <t>Bill card shows SHIP BY = "Flash Express" (saved; form closes back to read-only)</t>
   </si>
   <si>
-    <t>Order with status "Create Order"</t>
+    <t>Same seeded order as UD-bill (Create Order state)</t>
   </si>
   <si>
     <t>TS-03_TC-02</t>
@@ -575,7 +575,7 @@
     <t>Order Item shows "Quantity 5 item"</t>
   </si>
   <si>
-    <t>Any order</t>
+    <t>Same seeded order as UD-bill</t>
   </si>
   <si>
     <t>TS-03_TC-03</t>
@@ -690,7 +690,7 @@
     <t>Quantity stays at 1 (− button is disabled at value 1; the only way to remove is the trash icon). No maximum cap; quantity is not bound to stock (ordering above stock is allowed and later shows Out of Stock). [PO ORD-Q2]</t>
   </si>
   <si>
-    <t>Order with status "Create Order" (before Approved)</t>
+    <t>API seed: seedOrder(SEED_ORDER) — fresh order in Create Order state (before Approved); open via the seeded orderId. (Cancel itself is the teardown — order ends in Cancel state.)</t>
   </si>
   <si>
     <t>TA-02_TC-02</t>
@@ -702,7 +702,7 @@
     <t>Open detail → tap the "Cancel" button (yellow) → confirm in the dialog</t>
   </si>
   <si>
-    <t>Order: status Create Order</t>
+    <t>Order: &lt;seeded orderId&gt;, status Create Order</t>
   </si>
   <si>
     <t>(before Confirm) a confirmation dialog "ยืนยันการยกเลิกคำสั่งซื้อ ___ ?" with Confirm/Cancel buttons · (after Confirm) order changes to status "Cancel" (terminal, no further edits). If the order was already Picked, stock is returned. [PO ORD-Q9]</t>
@@ -718,7 +718,7 @@
 2. Cancel blocked after Approved (BUG)</t>
   </si>
   <si>
-    <t>Order with status "Request Approved" (already submitted)</t>
+    <t>API seed: seedOrder(SEED_ORDER) → advanceOrder(OS001) → advanceOrder(OS003) — fresh order advanced to Request Approved; open via the seeded orderId (no pre-existing data). Teardown: CancelOrder.</t>
   </si>
   <si>
     <t>TA-03_TC-01</t>
@@ -730,13 +730,13 @@
     <t>Open detail → look for the pencil on the Bill card and ORDER ITEMS</t>
   </si>
   <si>
-    <t>Order: ORD260610-00001 (Request Approved)</t>
+    <t>Order: &lt;seeded orderId&gt; (Request Approved, OS003)</t>
   </si>
   <si>
     <t>No pencil on the Bill card or ORDER ITEMS (not editable) · the Title pencil is still present</t>
   </si>
   <si>
-    <t>Order with current step = "ได้รับการอนุมัติ" (Approved)</t>
+    <t>Same seeded order as UD-lock (seedOrder(SEED_ORDER) → advanceOrder OS001 → OS003 = Request Approved). No pre-existing data. Teardown: CancelOrder.</t>
   </si>
   <si>
     <t>TA-03_TC-02</t>
@@ -746,9 +746,6 @@
   </si>
   <si>
     <t>Open detail → check whether the Cancel button is present</t>
-  </si>
-  <si>
-    <t>Order: ORD260610-00001</t>
   </si>
   <si>
     <t>Expected: the Cancel button should be hidden/blocked once the order is Approved (Cancel is only allowed before Approved). The button currently still appears at the Approved step → this is a BUG; expected to FAIL → open a defect. [PO ORD-Q5]</t>
@@ -791,7 +788,7 @@
 2. Search by part name (no filter — BUG)</t>
   </si>
   <si>
-    <t>Multiple orders including ORD260609-00001</t>
+    <t>API seed: 2 orders — seedOrder(SEED_ORDER) + seedOrder(SEED_ORDER_OOS) — so a specific seeded orderId exists to search for (no hard-coded pre-existing ID). Teardown: CancelOrder.</t>
   </si>
   <si>
     <t>TA-05_TC-01</t>
@@ -800,16 +797,16 @@
     <t>Search by Order ID (BUG: does not filter)</t>
   </si>
   <si>
-    <t>Type an Order ID in the Search box → tap Search</t>
-  </si>
-  <si>
-    <t>ORD260609-00001</t>
-  </si>
-  <si>
-    <t>Expected: list filters to only ORD260609-00001 (Search should filter by Order ID per placeholder "Search request ID or part..."). Actual: returns all orders (no filtering) → expected to FAIL → open a defect. [PO ORD-Q7]</t>
-  </si>
-  <si>
-    <t>An order containing item "iPhone 17 Pro Screen" plus other orders without it</t>
+    <t>Type the seeded Order ID in the Search box → tap Search</t>
+  </si>
+  <si>
+    <t>&lt;seeded orderId&gt;</t>
+  </si>
+  <si>
+    <t>Expected: list filters to only the searched Order ID (Search should filter by Order ID per placeholder "Search request ID or part..."). Actual: returns all orders (no filtering) → expected to FAIL → open a defect. [PO ORD-Q7]</t>
+  </si>
+  <si>
+    <t>Same seeded orders as TL-sid (SEED_ORDER_OOS contains iPhone 17 Pro Screen) plus other orders without it</t>
   </si>
   <si>
     <t>TA-05_TC-02</t>
@@ -836,7 +833,7 @@
     <t>1. Non-PIC user → Advance button hidden</t>
   </si>
   <si>
-    <t>Logged in as a user NOT in the PIC list of the current step</t>
+    <t>API seed: seedOrder(SEED_ORDER) — fresh order; then log in with a non-PIC account (ORD_NON_PIC_USERNAME/PASSWORD; PIC roles = Warehouse Approver / Manager). Teardown: CancelOrder.</t>
   </si>
   <si>
     <t>TA-06_TC-01</t>
@@ -3821,10 +3818,10 @@
         <v>238</v>
       </c>
       <c r="M35" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="N35" s="19" t="s">
         <v>239</v>
-      </c>
-      <c r="N35" s="19" t="s">
-        <v>240</v>
       </c>
       <c r="O35" s="19" t="s">
         <v>46</v>
@@ -3865,22 +3862,22 @@
         <v>34</v>
       </c>
       <c r="D36" s="19" t="s">
+        <v>240</v>
+      </c>
+      <c r="E36" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="E36" s="19" t="s">
+      <c r="F36" s="19" t="s">
         <v>242</v>
       </c>
-      <c r="F36" s="19" t="s">
+      <c r="G36" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="G36" s="19" t="s">
+      <c r="H36" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="H36" s="19" t="s">
+      <c r="I36" s="19" t="s">
         <v>245</v>
-      </c>
-      <c r="I36" s="19" t="s">
-        <v>246</v>
       </c>
       <c r="J36" s="19" t="s">
         <v>207</v>
@@ -3889,13 +3886,13 @@
         <v>42</v>
       </c>
       <c r="L36" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="M36" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="M36" s="19" t="s">
+      <c r="N36" s="19" t="s">
         <v>248</v>
-      </c>
-      <c r="N36" s="19" t="s">
-        <v>249</v>
       </c>
       <c r="O36" s="19" t="s">
         <v>46</v>
@@ -3936,22 +3933,22 @@
         <v>34</v>
       </c>
       <c r="D37" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="E37" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="E37" s="19" t="s">
+      <c r="F37" s="19" t="s">
         <v>251</v>
       </c>
-      <c r="F37" s="19" t="s">
+      <c r="G37" s="19" t="s">
         <v>252</v>
       </c>
-      <c r="G37" s="19" t="s">
+      <c r="H37" s="19" t="s">
         <v>253</v>
       </c>
-      <c r="H37" s="19" t="s">
+      <c r="I37" s="19" t="s">
         <v>254</v>
-      </c>
-      <c r="I37" s="19" t="s">
-        <v>255</v>
       </c>
       <c r="J37" s="19" t="s">
         <v>207</v>
@@ -3960,13 +3957,13 @@
         <v>42</v>
       </c>
       <c r="L37" s="19" t="s">
+        <v>255</v>
+      </c>
+      <c r="M37" s="19" t="s">
         <v>256</v>
       </c>
-      <c r="M37" s="19" t="s">
+      <c r="N37" s="19" t="s">
         <v>257</v>
-      </c>
-      <c r="N37" s="19" t="s">
-        <v>258</v>
       </c>
       <c r="O37" s="19" t="s">
         <v>46</v>
@@ -4007,22 +4004,22 @@
         <v>34</v>
       </c>
       <c r="D38" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="E38" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="E38" s="19" t="s">
+      <c r="F38" s="19" t="s">
         <v>251</v>
       </c>
-      <c r="F38" s="19" t="s">
-        <v>252</v>
-      </c>
       <c r="G38" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="H38" s="19" t="s">
         <v>259</v>
       </c>
-      <c r="H38" s="19" t="s">
+      <c r="I38" s="19" t="s">
         <v>260</v>
-      </c>
-      <c r="I38" s="19" t="s">
-        <v>261</v>
       </c>
       <c r="J38" s="19" t="s">
         <v>207</v>
@@ -4031,13 +4028,13 @@
         <v>42</v>
       </c>
       <c r="L38" s="19" t="s">
+        <v>261</v>
+      </c>
+      <c r="M38" s="19" t="s">
         <v>262</v>
       </c>
-      <c r="M38" s="19" t="s">
+      <c r="N38" s="19" t="s">
         <v>263</v>
-      </c>
-      <c r="N38" s="19" t="s">
-        <v>264</v>
       </c>
       <c r="O38" s="19" t="s">
         <v>46</v>
@@ -4078,22 +4075,22 @@
         <v>34</v>
       </c>
       <c r="D39" s="19" t="s">
+        <v>264</v>
+      </c>
+      <c r="E39" s="19" t="s">
         <v>265</v>
       </c>
-      <c r="E39" s="19" t="s">
+      <c r="F39" s="19" t="s">
         <v>266</v>
       </c>
-      <c r="F39" s="19" t="s">
+      <c r="G39" s="19" t="s">
         <v>267</v>
       </c>
-      <c r="G39" s="19" t="s">
+      <c r="H39" s="19" t="s">
         <v>268</v>
       </c>
-      <c r="H39" s="19" t="s">
+      <c r="I39" s="19" t="s">
         <v>269</v>
-      </c>
-      <c r="I39" s="19" t="s">
-        <v>270</v>
       </c>
       <c r="J39" s="19" t="s">
         <v>207</v>
@@ -4102,13 +4099,13 @@
         <v>42</v>
       </c>
       <c r="L39" s="19" t="s">
+        <v>270</v>
+      </c>
+      <c r="M39" s="19" t="s">
         <v>271</v>
       </c>
-      <c r="M39" s="19" t="s">
+      <c r="N39" s="19" t="s">
         <v>272</v>
-      </c>
-      <c r="N39" s="19" t="s">
-        <v>273</v>
       </c>
       <c r="O39" s="19" t="s">
         <v>46</v>

</xml_diff>